<commit_message>
chore: update maintenance fee calculator from latest table (v2)
</commit_message>
<xml_diff>
--- a/docs/Площи - Премиум Естейт V2.xlsx
+++ b/docs/Площи - Премиум Естейт V2.xlsx
@@ -1992,12 +1992,12 @@
         <v>16</v>
       </c>
       <c r="J7" s="5">
-        <f>'Жилищна част'!E337*7+'Жилищна част'!E340*3</f>
-        <v>1320</v>
+        <f>('Жилищна част'!E337*7+'Жилищна част'!E340*3)/1.2</f>
+        <v>1100</v>
       </c>
       <c r="K7" s="4">
         <f t="shared" si="1"/>
-        <v>1320</v>
+        <v>1100</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="3" t="s">
@@ -2033,7 +2033,8 @@
         <v>16</v>
       </c>
       <c r="J8" s="4">
-        <v>7185.80631966458</v>
+        <f>7185.80631966458/1.2</f>
+        <v>5988.171933</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>16</v>
@@ -2075,11 +2076,12 @@
         <v>1500</v>
       </c>
       <c r="J9" s="5">
-        <v>1740.0</v>
+        <f>1740/1.2</f>
+        <v>1450</v>
       </c>
       <c r="K9" s="4">
         <f t="shared" ref="K9:K13" si="3">J9</f>
-        <v>1740</v>
+        <v>1450</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="3" t="s">
@@ -2116,12 +2118,12 @@
         <v>650</v>
       </c>
       <c r="J10" s="5">
-        <f>2*960</f>
-        <v>1920</v>
+        <f>2*960/1.2</f>
+        <v>1600</v>
       </c>
       <c r="K10" s="4">
         <f t="shared" si="3"/>
-        <v>1920</v>
+        <v>1600</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="3" t="s">
@@ -2159,11 +2161,12 @@
         <v>400</v>
       </c>
       <c r="J11" s="5">
-        <v>690.0</v>
+        <f>690/1.2</f>
+        <v>575</v>
       </c>
       <c r="K11" s="4">
         <f t="shared" si="3"/>
-        <v>690</v>
+        <v>575</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="3" t="s">
@@ -2429,11 +2432,11 @@
       </c>
       <c r="J17" s="8">
         <f t="shared" si="8"/>
-        <v>14270.82632</v>
+        <v>12128.19193</v>
       </c>
       <c r="K17" s="8">
         <f t="shared" si="8"/>
-        <v>7085.02</v>
+        <v>6140.02</v>
       </c>
       <c r="L17" s="8">
         <f>L19+L20</f>
@@ -2492,11 +2495,11 @@
       </c>
       <c r="J19" s="10">
         <f t="shared" si="10"/>
-        <v>9615.80632</v>
+        <v>8013.171933</v>
       </c>
       <c r="K19" s="10">
         <f t="shared" si="10"/>
-        <v>2430</v>
+        <v>2025</v>
       </c>
       <c r="L19" s="10">
         <f>L23*'Жилищна част'!E335</f>
@@ -2538,11 +2541,11 @@
       </c>
       <c r="J20" s="10">
         <f t="shared" si="12"/>
-        <v>1920</v>
+        <v>1600</v>
       </c>
       <c r="K20" s="10">
         <f t="shared" si="12"/>
-        <v>1920</v>
+        <v>1600</v>
       </c>
       <c r="L20" s="10">
         <f>L24*'Жилищна част'!E336</f>
@@ -2584,11 +2587,11 @@
       </c>
       <c r="J21" s="10">
         <f t="shared" ref="J21:K21" si="15">SUM(J13,J15,J16,J14,J7)</f>
-        <v>2735.02</v>
+        <v>2515.02</v>
       </c>
       <c r="K21" s="10">
         <f t="shared" si="15"/>
-        <v>2735.02</v>
+        <v>2515.02</v>
       </c>
       <c r="L21" s="10"/>
       <c r="M21" s="9"/>
@@ -2637,11 +2640,11 @@
       </c>
       <c r="J23" s="14">
         <f>J19/'Жилищна част'!$E$335+J21/('Жилищна част'!$E$335+'Жилищна част'!$E$336)</f>
-        <v>0.7073693749</v>
+        <v>0.6010945923</v>
       </c>
       <c r="K23" s="14">
         <f>K19/'Жилищна част'!$E$335+K21/('Жилищна част'!$E$335+'Жилищна част'!$E$336)</f>
-        <v>0.2794631556</v>
+        <v>0.2445060762</v>
       </c>
       <c r="L23" s="15">
         <v>0.9</v>
@@ -2683,11 +2686,11 @@
       </c>
       <c r="J24" s="16">
         <f>(J20)/'Жилищна част'!$E$336+J21/('Жилищна част'!$E$336+'Жилищна част'!$E$335)</f>
-        <v>0.6829222017</v>
+        <v>0.580721948</v>
       </c>
       <c r="K24" s="16">
         <f>(K20)/'Жилищна част'!$E$336+K21/('Жилищна част'!$E$336+'Жилищна част'!$E$335)</f>
-        <v>0.6829222017</v>
+        <v>0.580721948</v>
       </c>
       <c r="L24" s="15">
         <v>0.5</v>
@@ -2725,11 +2728,11 @@
       </c>
       <c r="J25" s="11">
         <f>J24*'Жилищна част'!$E$336 + J23*'Жилищна част'!$E$335</f>
-        <v>14270.82632</v>
+        <v>12128.19193</v>
       </c>
       <c r="K25" s="11">
         <f>K24*'Жилищна част'!$E$336 + K23*'Жилищна част'!$E$335</f>
-        <v>7085.02</v>
+        <v>6140.02</v>
       </c>
       <c r="L25" s="11">
         <f>L24*'Жилищна част'!$E$336 + L23*'Жилищна част'!$E$335</f>

</xml_diff>

<commit_message>
feat: update fees and add PR preview video workflow
</commit_message>
<xml_diff>
--- a/docs/Площи - Премиум Естейт V2.xlsx
+++ b/docs/Площи - Премиум Естейт V2.xlsx
@@ -41,10 +41,10 @@
     <t>Общ Дом (без портиер)</t>
   </si>
   <si>
-    <t>“ГАБРИЕЛА МЕНИДЖМЪНТ” (24ч портиер)</t>
-  </si>
-  <si>
-    <t>“ГАБРИЕЛА МЕНИДЖМЪНТ” ЕООД (без портиер)</t>
+    <t>Габриела Мениджмънт (24ч портиер)</t>
+  </si>
+  <si>
+    <t>Габриела Мениджмънт (без портиер)</t>
   </si>
   <si>
     <t>Премиум Естейт</t>

</xml_diff>